<commit_message>
Implement Path 1 — evidence-tuned scoring model (v0.3)
- Re-weight categories (Skills 0.34, Profile 0.24, Avail/Ret 0.22, Mobility 0.12, Credibility 0.08)
- Convert feasibility items (language, relocation, travel, work-mode) to pass/review/unknown GATES
- Merge weak distinction signals (awards+authority+competition) into one "recognition" sub-criterion
- Add fairness flags (employer prestige, school prestige, tenure age-proxy, location adverse-impact)
- Redefine probability-to-stay via job-embeddedness proxies
- Engine: gate handling + feasibility section; report renders gates & fairness flags
- Tuning sheet + sync updated to exclude gates from weight sums

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/engine/tuning/Scoring_Model_Tuning.xlsx
+++ b/engine/tuning/Scoring_Model_Tuning.xlsx
@@ -129,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -159,6 +159,7 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -546,7 +547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -612,7 +613,7 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>0.22</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="8">
@@ -622,7 +623,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>0.3</v>
+        <v>0.34</v>
       </c>
     </row>
     <row r="9">
@@ -632,7 +633,7 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>0.13</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="10">
@@ -642,7 +643,7 @@
         </is>
       </c>
       <c r="B10" s="7" t="n">
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
     </row>
     <row r="11">
@@ -652,7 +653,7 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>0.15</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="12">
@@ -736,11 +737,11 @@
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>Employers – Key OEM: list &amp; relevance of companies worked at</t>
+          <t>Relevant domain experience — companies/OEMs worked at (relevance, not prestige)</t>
         </is>
       </c>
       <c r="C18" s="7" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="D18" s="12">
         <f>$B$7*C18*100</f>
@@ -763,7 +764,7 @@
         </is>
       </c>
       <c r="C19" s="7" t="n">
-        <v>0.25</v>
+        <v>0.3</v>
       </c>
       <c r="D19" s="12">
         <f>$B$7*C19*100</f>
@@ -786,7 +787,7 @@
         </is>
       </c>
       <c r="C20" s="7" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="D20" s="12">
         <f>$B$7*C20*100</f>
@@ -809,7 +810,7 @@
         </is>
       </c>
       <c r="C21" s="7" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="D21" s="12">
         <f>$B$7*C21*100</f>
@@ -836,7 +837,7 @@
         </is>
       </c>
       <c r="C22" s="7" t="n">
-        <v>0.1</v>
+        <v>0.25</v>
       </c>
       <c r="D22" s="12">
         <f>$B$7*C22*100</f>
@@ -898,7 +899,7 @@
         </is>
       </c>
       <c r="C26" s="7" t="n">
-        <v>0.4</v>
+        <v>0.45</v>
       </c>
       <c r="D26" s="12">
         <f>$B$8*C26*100</f>
@@ -921,7 +922,7 @@
         </is>
       </c>
       <c r="C27" s="7" t="n">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
       <c r="D27" s="12">
         <f>$B$8*C27*100</f>
@@ -944,7 +945,7 @@
         </is>
       </c>
       <c r="C28" s="7" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="D28" s="12">
         <f>$B$8*C28*100</f>
@@ -963,11 +964,11 @@
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>Language proficiency analysis</t>
+          <t>Professional associations, certifications and credentials</t>
         </is>
       </c>
       <c r="C29" s="7" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="D29" s="12">
         <f>$B$8*C29*100</f>
@@ -986,11 +987,11 @@
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>Professional associations, certifications and credentials</t>
-        </is>
-      </c>
-      <c r="C30" s="7" t="n">
-        <v>0.1</v>
+          <t>Language proficiency (role requirement)</t>
+        </is>
+      </c>
+      <c r="C30" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="D30" s="12">
         <f>$B$8*C30*100</f>
@@ -998,10 +999,14 @@
       </c>
       <c r="E30" s="13" t="inlineStr">
         <is>
-          <t>✅ now</t>
-        </is>
-      </c>
-      <c r="F30" s="14" t="inlineStr"/>
+          <t>🚪 gate</t>
+        </is>
+      </c>
+      <c r="F30" s="14" t="inlineStr">
+        <is>
+          <t>Feasibility gate — pass/review/unknown, not weighted</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="B31" s="8" t="inlineStr">
@@ -1023,20 +1028,20 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="19" t="inlineStr">
+      <c r="A33" s="20" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B33" s="19" t="inlineStr">
+      <c r="B33" s="20" t="inlineStr">
         <is>
           <t>3. Credibility, Reputation &amp; Distinction   (category weight in B9)</t>
         </is>
       </c>
-      <c r="C33" s="20" t="n"/>
-      <c r="D33" s="20" t="n"/>
-      <c r="E33" s="20" t="n"/>
-      <c r="F33" s="20" t="n"/>
+      <c r="C33" s="21" t="n"/>
+      <c r="D33" s="21" t="n"/>
+      <c r="E33" s="21" t="n"/>
+      <c r="F33" s="21" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="6" t="n">
@@ -1044,11 +1049,11 @@
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>Awards, distinctions, scholarships, honors, recognitions, alumni</t>
+          <t>Publications and patents (work-sample evidence of capability)</t>
         </is>
       </c>
       <c r="C34" s="7" t="n">
-        <v>0.3</v>
+        <v>0.45</v>
       </c>
       <c r="D34" s="12">
         <f>$B$9*C34*100</f>
@@ -1067,11 +1072,11 @@
       </c>
       <c r="B35" s="11" t="inlineStr">
         <is>
-          <t>References, feedback</t>
+          <t>Recognition: awards/honors, demonstrated authority (speaker/panel/committee), competitions</t>
         </is>
       </c>
       <c r="C35" s="7" t="n">
-        <v>0.2</v>
+        <v>0.35</v>
       </c>
       <c r="D35" s="12">
         <f>$B$9*C35*100</f>
@@ -1079,14 +1084,10 @@
       </c>
       <c r="E35" s="13" t="inlineStr">
         <is>
-          <t>⏳ later</t>
-        </is>
-      </c>
-      <c r="F35" s="14" t="inlineStr">
-        <is>
-          <t>reference checks / recruiter feedback input</t>
-        </is>
-      </c>
+          <t>✅ now</t>
+        </is>
+      </c>
+      <c r="F35" s="14" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="6" t="n">
@@ -1094,7 +1095,7 @@
       </c>
       <c r="B36" s="11" t="inlineStr">
         <is>
-          <t>Demonstrated expertise or domain authority: speaker, panel, trainer, committees</t>
+          <t>References, feedback</t>
         </is>
       </c>
       <c r="C36" s="7" t="n">
@@ -1106,103 +1107,107 @@
       </c>
       <c r="E36" s="13" t="inlineStr">
         <is>
+          <t>⏳ later</t>
+        </is>
+      </c>
+      <c r="F36" s="14" t="inlineStr">
+        <is>
+          <t>reference checks / recruiter feedback input (later stage)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>Sub-weights total</t>
+        </is>
+      </c>
+      <c r="C37" s="9">
+        <f>SUM(C34:C36)</f>
+        <v/>
+      </c>
+      <c r="D37" s="15">
+        <f>SUM(D34:D36)</f>
+        <v/>
+      </c>
+      <c r="E37" s="16">
+        <f>IF(ABS(C37-1)&lt;0.001,"✓","✗ fix=1.00")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="22" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B39" s="22" t="inlineStr">
+        <is>
+          <t>4. Availability &amp; Retention Potential   (category weight in B10)</t>
+        </is>
+      </c>
+      <c r="C39" s="23" t="n"/>
+      <c r="D39" s="23" t="n"/>
+      <c r="E39" s="23" t="n"/>
+      <c r="F39" s="23" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B40" s="11" t="inlineStr">
+        <is>
+          <t>Open to work or probability of being open to work (placeability)</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D40" s="12">
+        <f>$B$10*C40*100</f>
+        <v/>
+      </c>
+      <c r="E40" s="13" t="inlineStr">
+        <is>
           <t>✅ now</t>
         </is>
       </c>
-      <c r="F36" s="14" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B37" s="11" t="inlineStr">
-        <is>
-          <t>Competition: student club</t>
-        </is>
-      </c>
-      <c r="C37" s="7" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D37" s="12">
-        <f>$B$9*C37*100</f>
-        <v/>
-      </c>
-      <c r="E37" s="13" t="inlineStr">
+      <c r="F40" s="14" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B41" s="11" t="inlineStr">
+        <is>
+          <t>Tenure windows (current and avg. past) — retention proxy</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D41" s="12">
+        <f>$B$10*C41*100</f>
+        <v/>
+      </c>
+      <c r="E41" s="13" t="inlineStr">
         <is>
           <t>✅ now</t>
         </is>
       </c>
-      <c r="F37" s="14" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B38" s="11" t="inlineStr">
-        <is>
-          <t>Publications and patents</t>
-        </is>
-      </c>
-      <c r="C38" s="7" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="D38" s="12">
-        <f>$B$9*C38*100</f>
-        <v/>
-      </c>
-      <c r="E38" s="13" t="inlineStr">
-        <is>
-          <t>✅ now</t>
-        </is>
-      </c>
-      <c r="F38" s="14" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="B39" s="8" t="inlineStr">
-        <is>
-          <t>Sub-weights total</t>
-        </is>
-      </c>
-      <c r="C39" s="9">
-        <f>SUM(C34:C38)</f>
-        <v/>
-      </c>
-      <c r="D39" s="15">
-        <f>SUM(D34:D38)</f>
-        <v/>
-      </c>
-      <c r="E39" s="16">
-        <f>IF(ABS(C39-1)&lt;0.001,"✓","✗ fix=1.00")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="21" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B41" s="21" t="inlineStr">
-        <is>
-          <t>4. Availability &amp; Retention Potential   (category weight in B10)</t>
-        </is>
-      </c>
-      <c r="C41" s="22" t="n"/>
-      <c r="D41" s="22" t="n"/>
-      <c r="E41" s="22" t="n"/>
-      <c r="F41" s="22" t="n"/>
+      <c r="F41" s="14" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B42" s="11" t="inlineStr">
         <is>
-          <t>Interest in Kollabtek, clients &amp; sector companies (subscribed, connected, applied before)</t>
+          <t>Interest in Kollabtek, clients &amp; sector companies (engagement signals)</t>
         </is>
       </c>
       <c r="C42" s="7" t="n">
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
       <c r="D42" s="12">
         <f>$B$10*C42*100</f>
@@ -1221,15 +1226,15 @@
     </row>
     <row r="43">
       <c r="A43" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B43" s="11" t="inlineStr">
         <is>
-          <t>Open to work or probability of being open to work</t>
+          <t>Probability to stay — job-embeddedness proxies (community/location ties, tenure, local roots)</t>
         </is>
       </c>
       <c r="C43" s="7" t="n">
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="D43" s="12">
         <f>$B$10*C43*100</f>
@@ -1237,18 +1242,22 @@
       </c>
       <c r="E43" s="13" t="inlineStr">
         <is>
-          <t>✅ now</t>
-        </is>
-      </c>
-      <c r="F43" s="14" t="inlineStr"/>
+          <t>⏳ later</t>
+        </is>
+      </c>
+      <c r="F43" s="14" t="inlineStr">
+        <is>
+          <t>embeddedness proxies: location/region ties + retention model on past placements</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B44" s="11" t="inlineStr">
         <is>
-          <t>Contact analysis (recruiter, Kollabtek team)</t>
+          <t>Contact analysis (existing relationship, recruiter/Kollabtek team)</t>
         </is>
       </c>
       <c r="C44" s="7" t="n">
@@ -1270,101 +1279,101 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B45" s="11" t="inlineStr">
-        <is>
-          <t>Probabilities to stay at Kollabtek</t>
-        </is>
-      </c>
-      <c r="C45" s="7" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="D45" s="12">
-        <f>$B$10*C45*100</f>
-        <v/>
-      </c>
-      <c r="E45" s="13" t="inlineStr">
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>Sub-weights total</t>
+        </is>
+      </c>
+      <c r="C45" s="9">
+        <f>SUM(C40:C44)</f>
+        <v/>
+      </c>
+      <c r="D45" s="15">
+        <f>SUM(D40:D44)</f>
+        <v/>
+      </c>
+      <c r="E45" s="16">
+        <f>IF(ABS(C45-1)&lt;0.001,"✓","✗ fix=1.00")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="24" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B47" s="24" t="inlineStr">
+        <is>
+          <t>5. Mobility   (category weight in B11)</t>
+        </is>
+      </c>
+      <c r="C47" s="25" t="n"/>
+      <c r="D47" s="25" t="n"/>
+      <c r="E47" s="25" t="n"/>
+      <c r="F47" s="25" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B48" s="11" t="inlineStr">
+        <is>
+          <t>Location: proximity to role + local ties (embeddedness/retention proxy)</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="D48" s="12">
+        <f>$B$11*C48*100</f>
+        <v/>
+      </c>
+      <c r="E48" s="13" t="inlineStr">
+        <is>
+          <t>✅ now</t>
+        </is>
+      </c>
+      <c r="F48" s="14" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B49" s="11" t="inlineStr">
+        <is>
+          <t>Region – past and current studies and work (local-roots / embeddedness proxy)</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="D49" s="12">
+        <f>$B$11*C49*100</f>
+        <v/>
+      </c>
+      <c r="E49" s="13" t="inlineStr">
         <is>
           <t>⏳ later</t>
         </is>
       </c>
-      <c r="F45" s="14" t="inlineStr">
-        <is>
-          <t>retention model on past placements</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B46" s="11" t="inlineStr">
-        <is>
-          <t>Tenure windows (current and avg. past)</t>
-        </is>
-      </c>
-      <c r="C46" s="7" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="D46" s="12">
-        <f>$B$10*C46*100</f>
-        <v/>
-      </c>
-      <c r="E46" s="13" t="inlineStr">
-        <is>
-          <t>✅ now</t>
-        </is>
-      </c>
-      <c r="F46" s="14" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="B47" s="8" t="inlineStr">
-        <is>
-          <t>Sub-weights total</t>
-        </is>
-      </c>
-      <c r="C47" s="9">
-        <f>SUM(C42:C46)</f>
-        <v/>
-      </c>
-      <c r="D47" s="15">
-        <f>SUM(D42:D46)</f>
-        <v/>
-      </c>
-      <c r="E47" s="16">
-        <f>IF(ABS(C47-1)&lt;0.001,"✓","✗ fix=1.00")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="23" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B49" s="23" t="inlineStr">
-        <is>
-          <t>5. Mobility   (category weight in B11)</t>
-        </is>
-      </c>
-      <c r="C49" s="24" t="n"/>
-      <c r="D49" s="24" t="n"/>
-      <c r="E49" s="24" t="n"/>
-      <c r="F49" s="24" t="n"/>
+      <c r="F49" s="14" t="inlineStr">
+        <is>
+          <t>structured study/work region history (LinkedIn / enrichment)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B50" s="11" t="inlineStr">
         <is>
-          <t>Interest in relocation</t>
-        </is>
-      </c>
-      <c r="C50" s="7" t="n">
-        <v>0.2</v>
+          <t>Interest in relocation (feasibility)</t>
+        </is>
+      </c>
+      <c r="C50" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="D50" s="12">
         <f>$B$11*C50*100</f>
@@ -1372,22 +1381,26 @@
       </c>
       <c r="E50" s="13" t="inlineStr">
         <is>
-          <t>✅ now</t>
-        </is>
-      </c>
-      <c r="F50" s="14" t="inlineStr"/>
+          <t>🚪 gate</t>
+        </is>
+      </c>
+      <c r="F50" s="14" t="inlineStr">
+        <is>
+          <t>Feasibility gate — pass/review/unknown, not weighted</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B51" s="11" t="inlineStr">
         <is>
-          <t>Willingness to travel</t>
-        </is>
-      </c>
-      <c r="C51" s="7" t="n">
-        <v>0.15</v>
+          <t>Willingness to travel (feasibility)</t>
+        </is>
+      </c>
+      <c r="C51" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="D51" s="12">
         <f>$B$11*C51*100</f>
@@ -1395,22 +1408,26 @@
       </c>
       <c r="E51" s="13" t="inlineStr">
         <is>
-          <t>✅ now</t>
-        </is>
-      </c>
-      <c r="F51" s="14" t="inlineStr"/>
+          <t>🚪 gate</t>
+        </is>
+      </c>
+      <c r="F51" s="14" t="inlineStr">
+        <is>
+          <t>Feasibility gate — pass/review/unknown, not weighted</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B52" s="11" t="inlineStr">
         <is>
-          <t>Location: proximity to current role</t>
-        </is>
-      </c>
-      <c r="C52" s="7" t="n">
-        <v>0.3</v>
+          <t>Work mode: on-site, hybrid, remote (feasibility)</t>
+        </is>
+      </c>
+      <c r="C52" s="19" t="n">
+        <v>0</v>
       </c>
       <c r="D52" s="12">
         <f>$B$11*C52*100</f>
@@ -1418,92 +1435,46 @@
       </c>
       <c r="E52" s="13" t="inlineStr">
         <is>
-          <t>✅ now</t>
-        </is>
-      </c>
-      <c r="F52" s="14" t="inlineStr"/>
+          <t>🚪 gate</t>
+        </is>
+      </c>
+      <c r="F52" s="14" t="inlineStr">
+        <is>
+          <t>Feasibility gate — pass/review/unknown, not weighted</t>
+        </is>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B53" s="11" t="inlineStr">
-        <is>
-          <t>Region – past and current studies and work</t>
-        </is>
-      </c>
-      <c r="C53" s="7" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="D53" s="12">
-        <f>$B$11*C53*100</f>
-        <v/>
-      </c>
-      <c r="E53" s="13" t="inlineStr">
-        <is>
-          <t>⏳ later</t>
-        </is>
-      </c>
-      <c r="F53" s="14" t="inlineStr">
-        <is>
-          <t>structured study/work region history (LinkedIn / enrichment)</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B54" s="11" t="inlineStr">
-        <is>
-          <t>Work mode: on-site, hybrid, remote</t>
-        </is>
-      </c>
-      <c r="C54" s="7" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="D54" s="12">
-        <f>$B$11*C54*100</f>
-        <v/>
-      </c>
-      <c r="E54" s="13" t="inlineStr">
-        <is>
-          <t>✅ now</t>
-        </is>
-      </c>
-      <c r="F54" s="14" t="inlineStr"/>
+      <c r="B53" s="8" t="inlineStr">
+        <is>
+          <t>Sub-weights total</t>
+        </is>
+      </c>
+      <c r="C53" s="9">
+        <f>SUM(C48:C52)</f>
+        <v/>
+      </c>
+      <c r="D53" s="15">
+        <f>SUM(D48:D52)</f>
+        <v/>
+      </c>
+      <c r="E53" s="16">
+        <f>IF(ABS(C53-1)&lt;0.001,"✓","✗ fix=1.00")</f>
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="B55" s="8" t="inlineStr">
         <is>
-          <t>Sub-weights total</t>
-        </is>
-      </c>
-      <c r="C55" s="9">
-        <f>SUM(C50:C54)</f>
-        <v/>
+          <t>GRAND TOTAL — effective pts</t>
+        </is>
       </c>
       <c r="D55" s="15">
-        <f>SUM(D50:D54)</f>
+        <f>D23+D31+D37+D45+D53</f>
         <v/>
       </c>
       <c r="E55" s="16">
-        <f>IF(ABS(C55-1)&lt;0.001,"✓","✗ fix=1.00")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57">
-      <c r="B57" s="8" t="inlineStr">
-        <is>
-          <t>GRAND TOTAL — effective pts</t>
-        </is>
-      </c>
-      <c r="D57" s="15">
-        <f>D23+D31+D39+D47+D55</f>
-        <v/>
-      </c>
-      <c r="E57" s="16">
-        <f>IF(ABS(D57-100)&lt;0.1,"✓ =100","✗ check")</f>
+        <f>IF(ABS(D55-100)&lt;0.1,"✓ =100","✗ check")</f>
         <v/>
       </c>
     </row>
@@ -1516,7 +1487,7 @@
       <formula>ISNUMBER(SEARCH("✓",C12))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E17:E57">
+  <conditionalFormatting sqref="E17:E55">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>ISNUMBER(SEARCH("✗",E17))</formula>
     </cfRule>
@@ -1525,7 +1496,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="B7 B8 B9 B10 B11 C18 C19 C20 C21 C22 C26 C27 C28 C29 C30 C34 C35 C36 C37 C38 C42 C43 C44 C45 C46 C50 C51 C52 C53 C54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid weight" error="Weights must be between 0 and 1." type="decimal" operator="between">
+    <dataValidation sqref="B7 B8 B9 B10 B11 C18 C19 C20 C21 C22 C26 C27 C28 C29 C34 C35 C36 C40 C41 C42 C43 C44 C48 C49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid weight" error="Weights must be between 0 and 1." type="decimal" operator="between">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>

</xml_diff>